<commit_message>
feat: source weapon parameters from Excel and generated definitions (v0.31.4)
</commit_message>
<xml_diff>
--- a/tools/data_import/source/game_data.xlsx
+++ b/tools/data_import/source/game_data.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="R1185f3420ded42d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="R62049afbb32a4368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="Rb2ba77fd123e433d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="R3c6a0005747e4dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="R7764b260bbb6421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="Rd49112cd2c984d2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rf9396fa4ba46485b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="8" r:id="R2e9bed015fa446cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="Re76b5accca5446b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="R400e782cdc5c4037"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="Rde80e2b02d1a4f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="Rd5b42b7030ac4a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="Rf2feb8e50ed74666"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="Rd058dd564a2648c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rf400ca2987a84ee6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="8" r:id="R45354a2028364b3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,9 +68,6 @@
     <x:t xml:space="preserve">基础动力模块，为飞船提供主要推进力。</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">武器模块。类型专属参数：firepower。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">firepower</x:t>
   </x:si>
   <x:si>
@@ -225,7 +222,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="General"/>
+  </x:numFmts>
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -259,8 +259,19 @@
       <x:sz val="11"/>
       <x:name val="微软雅黑"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -282,6 +293,16 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -290,7 +311,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -320,6 +341,42 @@
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -1047,11 +1104,16 @@
     <x:col min="3" max="3" width="42" customWidth="1"/>
     <x:col min="4" max="8" width="14" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17" customHeight="1">
-      <x:c r="A1" s="7" t="s">
-        <x:v>17</x:v>
+      <x:c r="A1" s="7" t="str">
+        <x:v>武器模块。专属参数及单位见 README。</x:v>
       </x:c>
       <x:c r="B1" s="7"/>
       <x:c r="C1" s="7"/>
@@ -1060,6 +1122,21 @@
       <x:c r="F1" s="7"/>
       <x:c r="G1" s="7"/>
       <x:c r="H1" s="7"/>
+      <x:c r="J1" s="20" t="str">
+        <x:v>px</x:v>
+      </x:c>
+      <x:c r="K1" s="20" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="L1" s="20" t="str">
+        <x:v>deg/s</x:v>
+      </x:c>
+      <x:c r="M1" s="20" t="str">
+        <x:v>deg</x:v>
+      </x:c>
+      <x:c r="N1" s="20" t="str">
+        <x:v>px/s</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="12" customHeight="1">
       <x:c r="A2" s="1" t="s">
@@ -1084,21 +1161,36 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I2" s="11" t="str">
         <x:v>hp</x:v>
       </x:c>
+      <x:c r="J2" s="16" t="str">
+        <x:v>attack_range</x:v>
+      </x:c>
+      <x:c r="K2" s="16" t="str">
+        <x:v>fire_interval</x:v>
+      </x:c>
+      <x:c r="L2" s="16" t="str">
+        <x:v>turn_speed_degrees</x:v>
+      </x:c>
+      <x:c r="M2" s="16" t="str">
+        <x:v>fire_angle_tolerance_degrees</x:v>
+      </x:c>
+      <x:c r="N2" s="16" t="str">
+        <x:v>projectile_speed</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="C3" s="2" t="s">
         <x:v>20</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>21</x:v>
       </x:c>
       <x:c r="D3" s="2">
         <x:v>1</x:v>
@@ -1117,6 +1209,21 @@
       </x:c>
       <x:c r="I3" t="n">
         <x:v>20</x:v>
+      </x:c>
+      <x:c r="J3" s="23" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="K3" s="23" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="L3" s="23" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="M3" s="23" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N3" s="23" t="n">
+        <x:v>700</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1128,6 +1235,11 @@
       <x:c r="F4" s="2"/>
       <x:c r="G4" s="2"/>
       <x:c r="H4" s="2"/>
+      <x:c r="J4" s="23"/>
+      <x:c r="K4" s="23"/>
+      <x:c r="L4" s="23"/>
+      <x:c r="M4" s="23"/>
+      <x:c r="N4" s="23"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2"/>
@@ -1138,6 +1250,11 @@
       <x:c r="F5" s="2"/>
       <x:c r="G5" s="2"/>
       <x:c r="H5" s="2"/>
+      <x:c r="J5" s="23"/>
+      <x:c r="K5" s="23"/>
+      <x:c r="L5" s="23"/>
+      <x:c r="M5" s="23"/>
+      <x:c r="N5" s="23"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2"/>
@@ -1148,6 +1265,11 @@
       <x:c r="F6" s="2"/>
       <x:c r="G6" s="2"/>
       <x:c r="H6" s="2"/>
+      <x:c r="J6" s="23"/>
+      <x:c r="K6" s="23"/>
+      <x:c r="L6" s="23"/>
+      <x:c r="M6" s="23"/>
+      <x:c r="N6" s="23"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2"/>
@@ -1158,6 +1280,11 @@
       <x:c r="F7" s="2"/>
       <x:c r="G7" s="2"/>
       <x:c r="H7" s="2"/>
+      <x:c r="J7" s="23"/>
+      <x:c r="K7" s="23"/>
+      <x:c r="L7" s="23"/>
+      <x:c r="M7" s="23"/>
+      <x:c r="N7" s="23"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2"/>
@@ -1168,6 +1295,11 @@
       <x:c r="F8" s="2"/>
       <x:c r="G8" s="2"/>
       <x:c r="H8" s="2"/>
+      <x:c r="J8" s="23"/>
+      <x:c r="K8" s="23"/>
+      <x:c r="L8" s="23"/>
+      <x:c r="M8" s="23"/>
+      <x:c r="N8" s="23"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2"/>
@@ -1178,6 +1310,11 @@
       <x:c r="F9" s="2"/>
       <x:c r="G9" s="2"/>
       <x:c r="H9" s="2"/>
+      <x:c r="J9" s="23"/>
+      <x:c r="K9" s="23"/>
+      <x:c r="L9" s="23"/>
+      <x:c r="M9" s="23"/>
+      <x:c r="N9" s="23"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2"/>
@@ -1188,6 +1325,11 @@
       <x:c r="F10" s="2"/>
       <x:c r="G10" s="2"/>
       <x:c r="H10" s="2"/>
+      <x:c r="J10" s="23"/>
+      <x:c r="K10" s="23"/>
+      <x:c r="L10" s="23"/>
+      <x:c r="M10" s="23"/>
+      <x:c r="N10" s="23"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2"/>
@@ -1198,6 +1340,11 @@
       <x:c r="F11" s="2"/>
       <x:c r="G11" s="2"/>
       <x:c r="H11" s="2"/>
+      <x:c r="J11" s="23"/>
+      <x:c r="K11" s="23"/>
+      <x:c r="L11" s="23"/>
+      <x:c r="M11" s="23"/>
+      <x:c r="N11" s="23"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2"/>
@@ -1208,6 +1355,11 @@
       <x:c r="F12" s="2"/>
       <x:c r="G12" s="2"/>
       <x:c r="H12" s="2"/>
+      <x:c r="J12" s="23"/>
+      <x:c r="K12" s="23"/>
+      <x:c r="L12" s="23"/>
+      <x:c r="M12" s="23"/>
+      <x:c r="N12" s="23"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2"/>
@@ -1218,6 +1370,11 @@
       <x:c r="F13" s="2"/>
       <x:c r="G13" s="2"/>
       <x:c r="H13" s="2"/>
+      <x:c r="J13" s="23"/>
+      <x:c r="K13" s="23"/>
+      <x:c r="L13" s="23"/>
+      <x:c r="M13" s="23"/>
+      <x:c r="N13" s="23"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="2"/>
@@ -1228,6 +1385,11 @@
       <x:c r="F14" s="2"/>
       <x:c r="G14" s="2"/>
       <x:c r="H14" s="2"/>
+      <x:c r="J14" s="23"/>
+      <x:c r="K14" s="23"/>
+      <x:c r="L14" s="23"/>
+      <x:c r="M14" s="23"/>
+      <x:c r="N14" s="23"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="2"/>
@@ -1238,6 +1400,11 @@
       <x:c r="F15" s="2"/>
       <x:c r="G15" s="2"/>
       <x:c r="H15" s="2"/>
+      <x:c r="J15" s="23"/>
+      <x:c r="K15" s="23"/>
+      <x:c r="L15" s="23"/>
+      <x:c r="M15" s="23"/>
+      <x:c r="N15" s="23"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2"/>
@@ -1248,6 +1415,11 @@
       <x:c r="F16" s="2"/>
       <x:c r="G16" s="2"/>
       <x:c r="H16" s="2"/>
+      <x:c r="J16" s="23"/>
+      <x:c r="K16" s="23"/>
+      <x:c r="L16" s="23"/>
+      <x:c r="M16" s="23"/>
+      <x:c r="N16" s="23"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2"/>
@@ -1258,6 +1430,11 @@
       <x:c r="F17" s="2"/>
       <x:c r="G17" s="2"/>
       <x:c r="H17" s="2"/>
+      <x:c r="J17" s="23"/>
+      <x:c r="K17" s="23"/>
+      <x:c r="L17" s="23"/>
+      <x:c r="M17" s="23"/>
+      <x:c r="N17" s="23"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2"/>
@@ -1268,6 +1445,11 @@
       <x:c r="F18" s="2"/>
       <x:c r="G18" s="2"/>
       <x:c r="H18" s="2"/>
+      <x:c r="J18" s="23"/>
+      <x:c r="K18" s="23"/>
+      <x:c r="L18" s="23"/>
+      <x:c r="M18" s="23"/>
+      <x:c r="N18" s="23"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2"/>
@@ -1278,6 +1460,11 @@
       <x:c r="F19" s="2"/>
       <x:c r="G19" s="2"/>
       <x:c r="H19" s="2"/>
+      <x:c r="J19" s="23"/>
+      <x:c r="K19" s="23"/>
+      <x:c r="L19" s="23"/>
+      <x:c r="M19" s="23"/>
+      <x:c r="N19" s="23"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2"/>
@@ -1288,6 +1475,11 @@
       <x:c r="F20" s="2"/>
       <x:c r="G20" s="2"/>
       <x:c r="H20" s="2"/>
+      <x:c r="J20" s="23"/>
+      <x:c r="K20" s="23"/>
+      <x:c r="L20" s="23"/>
+      <x:c r="M20" s="23"/>
+      <x:c r="N20" s="23"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1310,7 +1502,7 @@
   <x:sheetData>
     <x:row r="1" ht="17" customHeight="1">
       <x:c r="A1" s="7" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B1" s="7"/>
       <x:c r="C1" s="7"/>
@@ -1343,7 +1535,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I2" s="11" t="str">
         <x:v>hp</x:v>
@@ -1351,13 +1543,13 @@
     </x:row>
     <x:row r="3" ht="15">
       <x:c r="A3" s="2" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="s">
+      <x:c r="C3" s="2" t="s">
         <x:v>25</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>26</x:v>
       </x:c>
       <x:c r="D3" s="2">
         <x:v>1</x:v>
@@ -1569,7 +1761,7 @@
   <x:sheetData>
     <x:row r="1" ht="17" customHeight="1">
       <x:c r="A1" s="7" t="s">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B1" s="7"/>
       <x:c r="C1" s="7"/>
@@ -1606,13 +1798,13 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="C3" s="2" t="s">
         <x:v>29</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>30</x:v>
       </x:c>
       <x:c r="D3" s="2">
         <x:v>1</x:v>
@@ -1804,7 +1996,7 @@
   <x:sheetData>
     <x:row r="1" ht="17" customHeight="1">
       <x:c r="A1" s="7" t="s">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B1" s="7"/>
       <x:c r="C1" s="7"/>
@@ -1841,13 +2033,13 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="C3" s="2" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>34</x:v>
       </x:c>
       <x:c r="D3" s="2">
         <x:v>2</x:v>
@@ -2035,58 +2227,58 @@
   <x:sheetData>
     <x:row r="1" ht="13.899999618530273">
       <x:c r="A1" s="1" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
         <x:v>35</x:v>
-      </x:c>
-      <x:c r="B1" s="1" t="s">
-        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B2" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="B2" t="s">
-        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B3" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="B3" t="s">
-        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B4" t="s">
         <x:v>41</x:v>
-      </x:c>
-      <x:c r="B4" t="s">
-        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B5" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="B5" t="s">
-        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B6" t="s">
         <x:v>45</x:v>
-      </x:c>
-      <x:c r="B6" t="s">
-        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B7" t="s">
         <x:v>47</x:v>
-      </x:c>
-      <x:c r="B7" t="s">
-        <x:v>48</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2104,39 +2296,39 @@
   <x:sheetData>
     <x:row r="1" ht="13.899999618530273">
       <x:c r="A1" s="3" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="s">
         <x:v>49</x:v>
-      </x:c>
-      <x:c r="B1" s="4" t="s">
-        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="13.899999618530273">
       <x:c r="A2" s="5" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="s">
         <x:v>51</x:v>
-      </x:c>
-      <x:c r="B2" s="6" t="s">
-        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="13.899999618530273">
       <x:c r="A3" s="5" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="s">
         <x:v>53</x:v>
-      </x:c>
-      <x:c r="B3" s="6" t="s">
-        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="13.899999618530273">
       <x:c r="A4" s="5" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
         <x:v>55</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="s">
-        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="13.899999618530273">
       <x:c r="A5" s="5" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
         <x:v>8</x:v>
@@ -2144,58 +2336,106 @@
     </x:row>
     <x:row r="6" ht="13.899999618530273">
       <x:c r="A6" s="5" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="13.899999618530273">
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="5" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="s">
-        <x:v>18</x:v>
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B7" s="24" t="str">
+        <x:v>firepower, attack_range, fire_interval, turn_speed_degrees, fire_angle_tolerance_degrees, projectile_speed</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="13.899999618530273">
       <x:c r="A8" s="5" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B8" s="6" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="13.899999618530273">
       <x:c r="A9" s="5" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
         <x:v>61</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="s">
-        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="13.899999618530273">
       <x:c r="A10" s="5" t="s">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B10" s="6" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="13.899999618530273">
       <x:c r="A11" s="5" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="s">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="B11" s="6" t="s">
-        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="13.899999618530273">
       <x:c r="A12" s="5" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="B12" s="6" t="s">
-        <x:v>67</x:v>
+    </x:row>
+    <x:row r="13" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A13" s="26" t="str">
+        <x:v>武器火力</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>firepower：每发初始伤害，必须 &gt; 0。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A14" s="26" t="str">
+        <x:v>攻击范围</x:v>
+      </x:c>
+      <x:c r="B14" s="27" t="str">
+        <x:v>attack_range：px，选敌范围及弹丸最大飞行距离，必须 &gt; 0。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A15" s="26" t="str">
+        <x:v>射击间隔</x:v>
+      </x:c>
+      <x:c r="B15" s="27" t="str">
+        <x:v>fire_interval：秒，两次射击的间隔，必须 &gt; 0；射速 = 1 / fire_interval。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A16" s="26" t="str">
+        <x:v>炮塔转速</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>turn_speed_degrees：度/秒，必须 &gt;= 0；0 表示不转动。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A17" s="26" t="str">
+        <x:v>瞄准容差</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>fire_angle_tolerance_degrees：度，允许开火的方向误差，范围 0~180。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A18" s="26" t="str">
+        <x:v>弹丸速度</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>projectile_speed：px/s，必须 &gt; 0；不另设弹丸寿命。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Restore Excel-driven module texture imports
</commit_message>
<xml_diff>
--- a/tools/data_import/source/game_data.xlsx
+++ b/tools/data_import/source/game_data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="R46b2889d04e74822"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="Rd5b9412c94094fb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="Rb78fd1dccee54abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="R5474e3fcb8104f18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="Re64a938d4d1e4222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="Rbdd6fb08ff394741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="R788ba61b3da84cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="Rd2bf0b9d3eca4484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="Rbbbc00b377cf4f76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="Rac627fa2963b4481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="R55aec1bf20dd48b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="R0232b93bd80249c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,15 +26,21 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="2">
@@ -44,15 +50,35 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -257,72 +283,79 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="52" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>id</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>display_name</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>width</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>height</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>mass</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>energy_cost</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>hp</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="6" t="str">
+        <x:v>texture_path</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
         <x:v>energy_output</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="12" t="str">
         <x:v>energy_smallreactor</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B2" s="12" t="str">
         <x:v>小型反应堆</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>基础能量模块，为飞船提供持续能量。</x:v>
       </x:c>
-      <x:c r="D2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="n">
+      <x:c r="D2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G2" t="n">
+      <x:c r="G2" s="12" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H2" t="n">
+      <x:c r="H2" s="12" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="I2" t="n">
+      <x:c r="I2" s="12" t="str">
+        <x:v>res://game/ship/art/modules/energy_smallreactor.png</x:v>
+      </x:c>
+      <x:c r="J2" s="12" t="n">
         <x:v>20</x:v>
       </x:c>
     </x:row>
@@ -335,72 +368,79 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="52" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>id</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>display_name</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>width</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>height</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>mass</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>energy_cost</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>hp</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="6" t="str">
+        <x:v>texture_path</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
         <x:v>thrust</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="12" t="str">
         <x:v>propulsion_smallengine</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B2" s="12" t="str">
         <x:v>小型引擎</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>基础动力模块，为飞船提供主要推进力。</x:v>
       </x:c>
-      <x:c r="D2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="n">
+      <x:c r="D2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G2" t="n">
+      <x:c r="G2" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H2" t="n">
+      <x:c r="H2" s="12" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="I2" t="n">
+      <x:c r="I2" s="12" t="str">
+        <x:v>res://game/ship/art/modules/propulsion_smallengine.png</x:v>
+      </x:c>
+      <x:c r="J2" s="12" t="n">
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -413,108 +453,122 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="52" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>id</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>display_name</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>width</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>height</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>mass</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>energy_cost</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>hp</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="6" t="str">
+        <x:v>texture_path</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
         <x:v>firepower</x:v>
       </x:c>
-      <x:c r="J1" s="4" t="str">
+      <x:c r="K1" s="6" t="str">
         <x:v>attack_range</x:v>
       </x:c>
-      <x:c r="K1" s="4" t="str">
+      <x:c r="L1" s="6" t="str">
         <x:v>fire_interval</x:v>
       </x:c>
-      <x:c r="L1" s="4" t="str">
+      <x:c r="M1" s="6" t="str">
         <x:v>turn_speed_degrees</x:v>
       </x:c>
-      <x:c r="M1" s="4" t="str">
+      <x:c r="N1" s="6" t="str">
         <x:v>projectile_speed</x:v>
       </x:c>
-      <x:c r="N1" s="4" t="str">
+      <x:c r="O1" s="6" t="str">
         <x:v>fire_angle_tolerance_degrees</x:v>
       </x:c>
+      <x:c r="P1" s="6" t="str">
+        <x:v>turret_texture_path</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="12" t="str">
         <x:v>weapon_cannon</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B2" s="12" t="str">
         <x:v>机炮</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>基础武器模块，提供稳定的常规火力。</x:v>
       </x:c>
-      <x:c r="D2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="n">
+      <x:c r="D2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G2" t="n">
+      <x:c r="G2" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H2" t="n">
+      <x:c r="H2" s="12" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="I2" t="n">
+      <x:c r="I2" s="12" t="str">
+        <x:v>res://game/ship/art/modules/weapon_cannon_base.png</x:v>
+      </x:c>
+      <x:c r="J2" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J2" t="n">
+      <x:c r="K2" s="12" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="K2" t="n">
+      <x:c r="L2" s="12" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="L2" t="n">
+      <x:c r="M2" s="12" t="n">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="M2" t="n">
+      <x:c r="N2" s="12" t="n">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="N2" t="n">
+      <x:c r="O2" s="12" t="n">
         <x:v>6</x:v>
+      </x:c>
+      <x:c r="P2" s="12" t="str">
+        <x:v>res://game/ship/art/modules/weapon_cannon_turret.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -526,72 +580,79 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="52" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>id</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>display_name</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>width</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>height</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>mass</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>energy_cost</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>hp</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="6" t="str">
+        <x:v>texture_path</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
         <x:v>protection</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="12" t="str">
         <x:v>defense_lightarmor</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B2" s="12" t="str">
         <x:v>轻型装甲</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>基础防护模块，为飞船提供结构防护。</x:v>
       </x:c>
-      <x:c r="D2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="n">
+      <x:c r="D2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G2" t="n">
+      <x:c r="G2" s="12" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H2" t="n">
+      <x:c r="H2" s="12" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="I2" t="n">
+      <x:c r="I2" s="12" t="str">
+        <x:v>res://game/ship/art/modules/defense_lightarmor.png</x:v>
+      </x:c>
+      <x:c r="J2" s="12" t="n">
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -604,66 +665,73 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>id</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>display_name</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>width</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>height</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>mass</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>energy_cost</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>hp</x:v>
       </x:c>
+      <x:c r="I1" s="6" t="str">
+        <x:v>texture_path</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="12" t="str">
         <x:v>function_radar</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B2" s="12" t="str">
         <x:v>雷达</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>基础功能模块。现阶段暂无额外参数。</x:v>
       </x:c>
-      <x:c r="D2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="n">
+      <x:c r="D2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G2" t="n">
+      <x:c r="G2" s="12" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="H2" t="n">
+      <x:c r="H2" s="12" t="n">
         <x:v>20</x:v>
+      </x:c>
+      <x:c r="I2" s="12" t="str">
+        <x:v>res://game/ship/art/modules/function_radar.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -675,66 +743,73 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>id</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>display_name</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>width</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>height</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>mass</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>energy_cost</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>hp</x:v>
       </x:c>
+      <x:c r="I1" s="6" t="str">
+        <x:v>texture_path</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="12" t="str">
         <x:v>core_bridge</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B2" s="12" t="str">
         <x:v>舰桥</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>飞船核心区域。核心模块被击毁时，飞船判定为沉没。</x:v>
       </x:c>
-      <x:c r="D2" t="n">
+      <x:c r="D2" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E2" t="n">
+      <x:c r="E2" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F2" t="n">
+      <x:c r="F2" s="12" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G2" t="n">
+      <x:c r="G2" s="12" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="H2" t="n">
+      <x:c r="H2" s="12" t="n">
         <x:v>20</x:v>
+      </x:c>
+      <x:c r="I2" s="12" t="str">
+        <x:v>res://game/ship/art/modules/core_bridge.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Use Chinese headers in game data workbook
</commit_message>
<xml_diff>
--- a/tools/data_import/source/game_data.xlsx
+++ b/tools/data_import/source/game_data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="Rc664de73d9c14951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="R6f1e66ef7ed441aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="R22dc82a3967a449b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="Rd673d66694fb4e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="Rfac5b201a8e248b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="R200930ce7b6548f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="R3f6d2e3fb0e14f45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="Rb1b8fd6064ed4bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="Ra463e464a044487c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="Rb515120481dc4b7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="R3402ef5d9ebc41de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="Rd3194a95d2ef43be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,7 +44,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -55,6 +55,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -257,40 +258,40 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="5.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="11.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="7.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>id</x:v>
+        <x:v>标识</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>display_name</x:v>
+        <x:v>显示名称</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>description</x:v>
+        <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>width</x:v>
+        <x:v>宽度</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>height</x:v>
+        <x:v>高度</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>energy_cost</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>texture_path</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>energy_output</x:v>
+        <x:v>能量输出</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -328,40 +329,40 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="5.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="5.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="4.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>id</x:v>
+        <x:v>标识</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>display_name</x:v>
+        <x:v>显示名称</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>description</x:v>
+        <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>width</x:v>
+        <x:v>宽度</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>height</x:v>
+        <x:v>高度</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>energy_cost</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>texture_path</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>thrust</x:v>
+        <x:v>推力</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -399,68 +400,68 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="5.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="8" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="9.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16.1299991607666" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="13.25" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="23.1299991607666" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="14.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="44" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15.25" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="9.75" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="11.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>id</x:v>
+        <x:v>标识</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>display_name</x:v>
+        <x:v>显示名称</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>description</x:v>
+        <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>width</x:v>
+        <x:v>宽度</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>height</x:v>
+        <x:v>高度</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>energy_cost</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>texture_path</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>firepower</x:v>
+        <x:v>火力</x:v>
       </x:c>
       <x:c r="I1" s="4" t="str">
-        <x:v>attack_range</x:v>
+        <x:v>攻击范围</x:v>
       </x:c>
       <x:c r="J1" s="4" t="str">
-        <x:v>fire_interval</x:v>
+        <x:v>射击间隔</x:v>
       </x:c>
       <x:c r="K1" s="4" t="str">
-        <x:v>turn_speed_degrees</x:v>
+        <x:v>炮塔转速（度/秒）</x:v>
       </x:c>
       <x:c r="L1" s="4" t="str">
-        <x:v>projectile_speed</x:v>
+        <x:v>弹速</x:v>
       </x:c>
       <x:c r="M1" s="4" t="str">
-        <x:v>fire_angle_tolerance_degrees</x:v>
+        <x:v>开火角容差（度）</x:v>
       </x:c>
       <x:c r="N1" s="4" t="str">
-        <x:v>firing_arc_degrees</x:v>
+        <x:v>射界（度）</x:v>
       </x:c>
       <x:c r="O1" s="4" t="str">
-        <x:v>turret_texture_path</x:v>
+        <x:v>炮塔贴图路径</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -519,44 +520,44 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="5.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="2.5" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="8.5" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="6" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="4.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>id</x:v>
+        <x:v>标识</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>display_name</x:v>
+        <x:v>显示名称</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>description</x:v>
+        <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>width</x:v>
+        <x:v>宽度</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>height</x:v>
+        <x:v>高度</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>energy_cost</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>texture_path</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>hp</x:v>
+        <x:v>生命值</x:v>
       </x:c>
       <x:c r="I1" s="4" t="str">
-        <x:v>protection</x:v>
+        <x:v>防护</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -597,36 +598,36 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="5.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>id</x:v>
+        <x:v>标识</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>display_name</x:v>
+        <x:v>显示名称</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>description</x:v>
+        <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>width</x:v>
+        <x:v>宽度</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>height</x:v>
+        <x:v>高度</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>energy_cost</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>texture_path</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -661,36 +662,36 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="5.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>id</x:v>
+        <x:v>标识</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>display_name</x:v>
+        <x:v>显示名称</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>description</x:v>
+        <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>width</x:v>
+        <x:v>宽度</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>height</x:v>
+        <x:v>高度</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>energy_cost</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>texture_path</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
     </x:row>
     <x:row r="2">

</xml_diff>